<commit_message>
Fill HSK1_parts_of_speech_7(301-350).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_7(301-350).xlsx
+++ b/HSK1_parts_of_speech_7(301-350).xlsx
@@ -601,6 +601,11 @@
           <t>мяч</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>мяч, шар; мяч/игра (足球, 打球)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +632,11 @@
           <t>идти</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>идти, ехать (куда-л.); уходить; вспомогательный глагол намерения (我去看看)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +663,16 @@
           <t>прошлый год</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>прошлый год</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>устойчивое словообразовательное сочетание: 去 + 年</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -679,6 +699,16 @@
           <t>жаркий, горячий</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>нагревать, греть (热一热菜); становиться жарким (天热了)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>жаркий, горячий (о погоде, воде)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -705,6 +735,11 @@
           <t>человек</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>человек, люди</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -731,6 +766,11 @@
           <t>знать (в лицо)</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>знать, быть знакомым; узнавать</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -757,6 +797,11 @@
           <t>ответственный</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>серьёзный, добросовестный, ответственный</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -783,6 +828,11 @@
           <t>день, дата</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>день; число, дата; солнце; день недели</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -809,6 +859,11 @@
           <t>дата</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>дата, число</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -835,6 +890,11 @@
           <t>мясо</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>мясо</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -861,6 +921,11 @@
           <t>три</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>три</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -887,6 +952,11 @@
           <t>гора</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>гора</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -913,6 +983,11 @@
           <t>торговый центр</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>торговый центр</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -939,6 +1014,11 @@
           <t>магазин</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>магазин</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -965,6 +1045,21 @@
           <t>наверху; верхний</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>верх, верхняя часть; прошлое</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>подниматься; идти на, подавать (上课, 上车)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>вышестоящий, предыдущий (上级, 上次)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -991,6 +1086,16 @@
           <t>выходить на работу</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>идти на работу, работать (о смене)</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 上 + 班 (上了一天的班)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1017,6 +1122,16 @@
           <t>верх, наверху</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>верх, верхняя сторона, наверху</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>локативное слово (方位词): 上 + 边</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1043,6 +1158,16 @@
           <t>садиться в машину</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>садиться в машину/транспорт</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>словосочетание (глагол + дополнение): 上 + 车</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1069,6 +1194,16 @@
           <t>прошлый раз</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>прошлый раз, предыдущий раз</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>устойчивое сочетание: 上 + 次</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1095,6 +1230,16 @@
           <t>посещать урок</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>идти на урок, посещать занятие; вести урок (об учителе)</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 上 + 课</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1121,6 +1266,16 @@
           <t>выходить в Интернет</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>выходить в Интернет</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 上 + 网</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1147,6 +1302,11 @@
           <t>до полудня</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>утро (примерно с 8 до 11 часов)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1173,6 +1333,16 @@
           <t>ходить в школу</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>ходить в школу, учиться (о школьнике/студенте)</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 上 + 学</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1199,6 +1369,16 @@
           <t>мало</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>уменьшать, экономить (少抽烟)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>мало, немногочисленный; молодой в летах</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1225,6 +1405,11 @@
           <t>кто</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>кто</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1251,6 +1436,16 @@
           <t>тело; на теле</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>тело; на теле; при себе (身上没钱)</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>локативная конструкция: 身 + 上</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1277,6 +1472,11 @@
           <t>тело</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>тело, здоровье</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1303,6 +1503,11 @@
           <t>что</t>
         </is>
       </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>что, какой (вопросительное/неопределённое)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1329,6 +1534,16 @@
           <t>заболеть</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>заболеть, быть больным</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 生 + 病 (生了很重的病)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1355,6 +1570,16 @@
           <t>разозлиться</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>сердиться, злиться</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 生 + 气</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1381,6 +1606,11 @@
           <t>день рождения</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>день рождения</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1407,6 +1637,11 @@
           <t>десять</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>десять</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1433,6 +1668,11 @@
           <t>время, во время</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>время, момент, «когда» (……的时候)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1459,6 +1699,11 @@
           <t>промежуток времени</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>время, промежуток времени</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1485,6 +1730,11 @@
           <t>дело</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>дело, событие</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1511,6 +1761,11 @@
           <t>пробовать</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>пробовать, испытывать</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1537,6 +1792,11 @@
           <t>быть, являться</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>быть, являться</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1563,6 +1823,11 @@
           <t>не так ли</t>
         </is>
       </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>грамматическая конструкция: вопросительная форма А не А? (是 + 不 + 是), отдельной частью речи не является</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1589,6 +1854,16 @@
           <t>рука</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>рука, кисть</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>для приёмов/умений (有两手 — «иметь козыри в рукаве»)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1615,6 +1890,11 @@
           <t>мобильный телефон</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>мобильный телефон</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1641,6 +1921,11 @@
           <t>книга</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>книга</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1667,6 +1952,11 @@
           <t>сумка для книг, школьный портфель</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>школьный рюкзак, сумка для книг</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1693,6 +1983,11 @@
           <t>книжный магазин</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>книжный магазин</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1719,6 +2014,11 @@
           <t>дерево</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>дерево</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1745,6 +2045,16 @@
           <t>вода</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>вода</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>для водных единиц ( редк.; обычно со счётным словом: 一杯水)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1771,6 +2081,11 @@
           <t>фрукты</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>фрукты</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1797,6 +2112,11 @@
           <t>спать, уснуть, засыпать</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>спать, засыпать</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1823,6 +2143,16 @@
           <t>спать, ложиться спать</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>спать, ложиться спать</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 睡 + 觉 (睡了个好觉)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1849,6 +2179,11 @@
           <t>говорить</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>говорить, сказать</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1873,6 +2208,16 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>говорить, рассказывать</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>говорить, беседовать</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词): 说 + 话</t>
         </is>
       </c>
     </row>

</xml_diff>